<commit_message>
Improve order status and follow-up rules
</commit_message>
<xml_diff>
--- a/data/sample_orders.xlsx
+++ b/data/sample_orders.xlsx
@@ -1249,7 +1249,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>placed</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1299,7 +1299,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>placed</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1349,7 +1349,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>placed</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1399,7 +1399,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>placed</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1449,7 +1449,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>placed</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1499,7 +1499,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>placed</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1549,7 +1549,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>placed</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1599,7 +1599,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>placed</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1649,7 +1649,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>placed</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1699,7 +1699,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>placed</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1749,7 +1749,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>placed</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1799,7 +1799,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>placed</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1849,7 +1849,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>placed</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1899,7 +1899,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>placed</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -1949,7 +1949,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>placed</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -1976,7 +1976,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-10-16 07:10:05</t>
+          <t>2026-10-16 08:55:14</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2022,7 +2022,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-10-16 07:10:05</t>
+          <t>2026-10-16 08:55:14</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-10-16 07:10:05</t>
+          <t>2026-10-16 08:55:14</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-10-16 07:10:05</t>
+          <t>2026-10-16 08:55:14</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-10-16 07:10:05</t>
+          <t>2026-10-16 08:55:14</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2206,7 +2206,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-10-16 07:10:05</t>
+          <t>2026-10-16 08:55:14</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2252,7 +2252,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-10-16 07:10:05</t>
+          <t>2026-10-16 08:55:14</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2298,7 +2298,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-10-16 07:10:05</t>
+          <t>2026-10-16 08:55:14</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2344,7 +2344,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-10-16 07:10:05</t>
+          <t>2026-10-16 08:55:14</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2390,7 +2390,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-10-16 07:10:05</t>
+          <t>2026-10-16 08:55:14</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2436,7 +2436,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-10-16 07:10:05</t>
+          <t>2026-10-16 08:55:14</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2482,7 +2482,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-10-16 07:10:05</t>
+          <t>2026-10-16 08:55:14</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2528,7 +2528,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-10-16 07:10:05</t>
+          <t>2026-10-16 08:55:14</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2574,7 +2574,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-10-16 07:10:05</t>
+          <t>2026-10-16 08:55:14</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2620,7 +2620,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-10-16 07:10:05</t>
+          <t>2026-10-16 08:55:14</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2666,7 +2666,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-10-15 17:10:05</t>
+          <t>2026-10-15 18:55:14</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2689,7 +2689,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>placed</t>
         </is>
       </c>
       <c r="H47" t="inlineStr"/>
@@ -2712,7 +2712,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-10-15 17:10:05</t>
+          <t>2026-10-15 18:55:14</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2735,7 +2735,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>placed</t>
         </is>
       </c>
       <c r="H48" t="inlineStr"/>
@@ -2758,7 +2758,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-10-15 17:10:05</t>
+          <t>2026-10-15 18:55:14</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2781,7 +2781,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>placed</t>
         </is>
       </c>
       <c r="H49" t="inlineStr"/>
@@ -2804,7 +2804,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-10-15 17:10:05</t>
+          <t>2026-10-15 18:55:14</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2827,7 +2827,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>placed</t>
         </is>
       </c>
       <c r="H50" t="inlineStr"/>
@@ -2850,7 +2850,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-10-15 17:10:05</t>
+          <t>2026-10-15 18:55:14</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2873,7 +2873,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>placed</t>
         </is>
       </c>
       <c r="H51" t="inlineStr"/>
@@ -2919,7 +2919,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>placed</t>
         </is>
       </c>
       <c r="H52" t="inlineStr"/>
@@ -2965,7 +2965,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>placed</t>
         </is>
       </c>
       <c r="H53" t="inlineStr"/>
@@ -3011,7 +3011,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>placed</t>
         </is>
       </c>
       <c r="H54" t="inlineStr"/>
@@ -3057,7 +3057,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>placed</t>
         </is>
       </c>
       <c r="H55" t="inlineStr"/>
@@ -3103,7 +3103,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>placed</t>
         </is>
       </c>
       <c r="H56" t="inlineStr"/>
@@ -3149,7 +3149,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>placed</t>
         </is>
       </c>
       <c r="H57" t="inlineStr"/>
@@ -3195,7 +3195,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>placed</t>
         </is>
       </c>
       <c r="H58" t="inlineStr"/>
@@ -3241,7 +3241,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>placed</t>
         </is>
       </c>
       <c r="H59" t="inlineStr"/>
@@ -3287,7 +3287,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>placed</t>
         </is>
       </c>
       <c r="H60" t="inlineStr"/>
@@ -3333,7 +3333,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>placed</t>
         </is>
       </c>
       <c r="H61" t="inlineStr"/>
@@ -3379,7 +3379,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>in transit</t>
+          <t>dispatched</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -3429,7 +3429,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>in transit</t>
+          <t>dispatched</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -3479,7 +3479,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>in transit</t>
+          <t>dispatched</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -3529,7 +3529,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>in transit</t>
+          <t>dispatched</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -3579,7 +3579,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>in transit</t>
+          <t>dispatched</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -3629,7 +3629,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>in transit</t>
+          <t>dispatched</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -3679,7 +3679,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>in transit</t>
+          <t>dispatched</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -3729,7 +3729,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>in transit</t>
+          <t>dispatched</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -3779,7 +3779,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>in transit</t>
+          <t>dispatched</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -3829,7 +3829,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>in transit</t>
+          <t>dispatched</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -3879,7 +3879,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>in transit</t>
+          <t>dispatched</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -3929,7 +3929,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>in transit</t>
+          <t>dispatched</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -3979,7 +3979,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>in transit</t>
+          <t>dispatched</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -4029,7 +4029,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>in transit</t>
+          <t>dispatched</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -4079,7 +4079,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>in transit</t>
+          <t>dispatched</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -4129,7 +4129,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>failed delivery</t>
+          <t>failed_delivery</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -4179,7 +4179,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>failed delivery</t>
+          <t>failed_delivery</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -4229,7 +4229,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>failed delivery</t>
+          <t>failed_delivery</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -4279,7 +4279,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>failed delivery</t>
+          <t>failed_delivery</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -4329,7 +4329,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>failed delivery</t>
+          <t>failed_delivery</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -4379,7 +4379,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>failed delivery</t>
+          <t>failed_delivery</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -4429,7 +4429,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>failed delivery</t>
+          <t>failed_delivery</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -4479,7 +4479,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>failed delivery</t>
+          <t>failed_delivery</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -4529,7 +4529,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>failed delivery</t>
+          <t>failed_delivery</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
@@ -4579,7 +4579,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>failed delivery</t>
+          <t>failed_delivery</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -4629,7 +4629,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>in transit</t>
+          <t>dispatched</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -4679,7 +4679,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>in transit</t>
+          <t>dispatched</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
@@ -4729,7 +4729,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>in transit</t>
+          <t>dispatched</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
@@ -4779,7 +4779,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>in transit</t>
+          <t>dispatched</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
@@ -4829,7 +4829,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>in transit</t>
+          <t>dispatched</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -4879,7 +4879,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>in transit</t>
+          <t>dispatched</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
@@ -4929,7 +4929,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>in transit</t>
+          <t>dispatched</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -4979,7 +4979,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>in transit</t>
+          <t>dispatched</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
@@ -5029,7 +5029,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>in transit</t>
+          <t>dispatched</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
@@ -5079,7 +5079,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>in transit</t>
+          <t>dispatched</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
@@ -5605,7 +5605,7 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>placed</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
@@ -5651,7 +5651,7 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>placed</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
@@ -5699,7 +5699,7 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>placed</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
@@ -5745,7 +5745,7 @@
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>placed</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
@@ -5770,7 +5770,11 @@
           <t>ORD-INVALID-005</t>
         </is>
       </c>
-      <c r="B111" t="inlineStr"/>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
       <c r="C111" t="inlineStr">
         <is>
           <t>Customer ORD-NORM-C-011</t>
@@ -5789,11 +5793,7 @@
           <t>Prepaid</t>
         </is>
       </c>
-      <c r="G111" t="inlineStr">
-        <is>
-          <t>confirmed</t>
-        </is>
-      </c>
+      <c r="G111" t="inlineStr"/>
       <c r="H111" t="inlineStr">
         <is>
           <t>2026-10-16</t>

</xml_diff>

<commit_message>
Improve auto date generating logic
</commit_message>
<xml_diff>
--- a/data/sample_orders.xlsx
+++ b/data/sample_orders.xlsx
@@ -476,7 +476,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-14 08:00:00</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -526,7 +526,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-14 08:00:00</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -576,7 +576,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-14 08:00:00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-14 08:00:00</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -676,7 +676,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-14 08:00:00</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -726,7 +726,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-14 08:00:00</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -776,7 +776,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-14 08:00:00</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -826,7 +826,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-14 08:00:00</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -876,7 +876,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-14 08:00:00</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -926,7 +926,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-14 08:00:00</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -976,7 +976,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-14 08:00:00</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1026,7 +1026,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-14 08:00:00</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1076,7 +1076,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-14 08:00:00</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1126,7 +1126,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-14 08:00:00</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1176,7 +1176,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-14 08:00:00</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1226,7 +1226,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-16 08:00:00</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1276,7 +1276,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-16 08:00:00</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1326,7 +1326,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-16 08:00:00</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1376,7 +1376,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-16 08:00:00</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1426,7 +1426,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-16 08:00:00</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1476,7 +1476,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-16 08:00:00</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1526,7 +1526,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-16 08:00:00</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1576,7 +1576,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-16 08:00:00</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1626,7 +1626,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-16 08:00:00</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1676,7 +1676,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-16 08:00:00</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1726,7 +1726,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-16 08:00:00</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-16 08:00:00</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-16 08:00:00</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1876,7 +1876,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-16 08:00:00</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-16 08:00:00</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1976,7 +1976,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-10-16 08:55:14</t>
+          <t>2026-10-16 09:01:26</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2022,7 +2022,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-10-16 08:55:14</t>
+          <t>2026-10-16 09:01:26</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-10-16 08:55:14</t>
+          <t>2026-10-16 09:01:26</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-10-16 08:55:14</t>
+          <t>2026-10-16 09:01:26</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-10-16 08:55:14</t>
+          <t>2026-10-16 09:01:26</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2206,7 +2206,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-10-16 08:55:14</t>
+          <t>2026-10-16 09:01:26</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2252,7 +2252,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-10-16 08:55:14</t>
+          <t>2026-10-16 09:01:26</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2298,7 +2298,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-10-16 08:55:14</t>
+          <t>2026-10-16 09:01:26</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2344,7 +2344,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-10-16 08:55:14</t>
+          <t>2026-10-16 09:01:26</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2390,7 +2390,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-10-16 08:55:14</t>
+          <t>2026-10-16 09:01:26</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2436,7 +2436,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-10-16 08:55:14</t>
+          <t>2026-10-16 09:01:26</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2482,7 +2482,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-10-16 08:55:14</t>
+          <t>2026-10-16 09:01:26</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2528,7 +2528,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-10-16 08:55:14</t>
+          <t>2026-10-16 09:01:26</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2574,7 +2574,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-10-16 08:55:14</t>
+          <t>2026-10-16 09:01:26</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2620,7 +2620,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-10-16 08:55:14</t>
+          <t>2026-10-16 09:01:26</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2666,7 +2666,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-10-15 18:55:14</t>
+          <t>2026-10-15 19:01:26</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2712,7 +2712,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-10-15 18:55:14</t>
+          <t>2026-10-15 19:01:26</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-10-15 18:55:14</t>
+          <t>2026-10-15 19:01:26</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2804,7 +2804,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-10-15 18:55:14</t>
+          <t>2026-10-15 19:01:26</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2850,7 +2850,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-10-15 18:55:14</t>
+          <t>2026-10-15 19:01:26</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -3356,7 +3356,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-12 08:00:00</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -3406,7 +3406,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-12 08:00:00</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3456,7 +3456,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-12 08:00:00</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3506,7 +3506,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-12 08:00:00</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3556,7 +3556,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-12 08:00:00</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -3606,7 +3606,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-12 08:00:00</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3656,7 +3656,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-12 08:00:00</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3706,7 +3706,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-12 08:00:00</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3756,7 +3756,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-12 08:00:00</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -3806,7 +3806,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-12 08:00:00</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -3856,7 +3856,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-12 08:00:00</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -3906,7 +3906,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-12 08:00:00</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -3956,7 +3956,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-12 08:00:00</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-12 08:00:00</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -4056,7 +4056,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-12 08:00:00</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -4106,7 +4106,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-14 08:00:00</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-14 08:00:00</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -4206,7 +4206,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-14 08:00:00</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -4256,7 +4256,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-14 08:00:00</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -4306,7 +4306,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-14 08:00:00</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -4356,7 +4356,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-14 08:00:00</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -4406,7 +4406,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-14 08:00:00</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -4456,7 +4456,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-14 08:00:00</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -4506,7 +4506,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-14 08:00:00</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -4556,7 +4556,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-14 08:00:00</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -4606,7 +4606,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-12 08:00:00</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -4656,7 +4656,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-12 08:00:00</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -4706,7 +4706,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-12 08:00:00</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -4756,7 +4756,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-12 08:00:00</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-12 08:00:00</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -4856,7 +4856,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-12 08:00:00</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -4906,7 +4906,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-12 08:00:00</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -4956,7 +4956,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-12 08:00:00</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -5006,7 +5006,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-12 08:00:00</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -5056,7 +5056,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-12 08:00:00</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -5106,7 +5106,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-14 08:00:00</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -5152,7 +5152,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-14 08:00:00</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -5198,7 +5198,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-14 08:00:00</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -5244,7 +5244,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-14 08:00:00</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -5290,7 +5290,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-14 08:00:00</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -5336,7 +5336,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-14 08:00:00</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -5386,7 +5386,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-14 08:00:00</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -5436,7 +5436,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-14 08:00:00</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -5486,7 +5486,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-14 08:00:00</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -5536,7 +5536,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-14 08:00:00</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -5586,7 +5586,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-16 08:00:00</t>
         </is>
       </c>
       <c r="C107" t="inlineStr"/>
@@ -5632,7 +5632,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-16 08:00:00</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -5678,7 +5678,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-16 08:00:00</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -5726,7 +5726,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-16 08:00:00</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -5772,7 +5772,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-16 08:00:00</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">

</xml_diff>

<commit_message>
implemented invalid order interception
</commit_message>
<xml_diff>
--- a/data/sample_orders.xlsx
+++ b/data/sample_orders.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J111"/>
+  <dimension ref="A1:J117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1976,7 +1976,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-10-16 09:01:26</t>
+          <t>2026-10-16 09:58:18</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2022,7 +2022,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-10-16 09:01:26</t>
+          <t>2026-10-16 09:58:18</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-10-16 09:01:26</t>
+          <t>2026-10-16 09:58:18</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-10-16 09:01:26</t>
+          <t>2026-10-16 09:58:18</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-10-16 09:01:26</t>
+          <t>2026-10-16 09:58:18</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2206,7 +2206,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-10-16 09:01:26</t>
+          <t>2026-10-16 09:58:18</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2252,7 +2252,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-10-16 09:01:26</t>
+          <t>2026-10-16 09:58:18</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2298,7 +2298,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-10-16 09:01:26</t>
+          <t>2026-10-16 09:58:18</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2344,7 +2344,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-10-16 09:01:26</t>
+          <t>2026-10-16 09:58:18</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2390,7 +2390,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-10-16 09:01:26</t>
+          <t>2026-10-16 09:58:18</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2436,7 +2436,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-10-16 09:01:26</t>
+          <t>2026-10-16 09:58:18</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2482,7 +2482,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-10-16 09:01:26</t>
+          <t>2026-10-16 09:58:18</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2528,7 +2528,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-10-16 09:01:26</t>
+          <t>2026-10-16 09:58:18</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2574,7 +2574,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-10-16 09:01:26</t>
+          <t>2026-10-16 09:58:18</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2620,7 +2620,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-10-16 09:01:26</t>
+          <t>2026-10-16 09:58:18</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2666,7 +2666,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-10-15 19:01:26</t>
+          <t>2026-10-15 19:58:18</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2712,7 +2712,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-10-15 19:01:26</t>
+          <t>2026-10-15 19:58:18</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-10-15 19:01:26</t>
+          <t>2026-10-15 19:58:18</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2804,7 +2804,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-10-15 19:01:26</t>
+          <t>2026-10-15 19:58:18</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2850,7 +2850,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-10-15 19:01:26</t>
+          <t>2026-10-15 19:58:18</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -5101,7 +5101,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>ORD-DATA-001</t>
+          <t>ORD-SHIP-EXTRA-001</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -5111,7 +5111,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Customer ORD-DATA-001</t>
+          <t>Customer ORD-SHIP-EXTRA-001</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -5137,7 +5137,11 @@
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="I97" t="inlineStr"/>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="J97" t="inlineStr">
         <is>
           <t>Ravi Kumar</t>
@@ -5147,7 +5151,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>ORD-DATA-002</t>
+          <t>ORD-SHIP-EXTRA-002</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -5157,7 +5161,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Customer ORD-DATA-002</t>
+          <t>Customer ORD-SHIP-EXTRA-002</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -5183,7 +5187,11 @@
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="I98" t="inlineStr"/>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="J98" t="inlineStr">
         <is>
           <t>Ravi Kumar</t>
@@ -5193,7 +5201,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>ORD-DATA-003</t>
+          <t>ORD-SHIP-EXTRA-003</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -5203,7 +5211,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Customer ORD-DATA-003</t>
+          <t>Customer ORD-SHIP-EXTRA-003</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -5229,7 +5237,11 @@
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="I99" t="inlineStr"/>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="J99" t="inlineStr">
         <is>
           <t>Ravi Kumar</t>
@@ -5239,7 +5251,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>ORD-DATA-004</t>
+          <t>ORD-SHIP-EXTRA-004</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -5249,7 +5261,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Customer ORD-DATA-004</t>
+          <t>Customer ORD-SHIP-EXTRA-004</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -5275,7 +5287,11 @@
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="I100" t="inlineStr"/>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="J100" t="inlineStr">
         <is>
           <t>Ravi Kumar</t>
@@ -5285,7 +5301,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>ORD-DATA-005</t>
+          <t>ORD-SHIP-EXTRA-005</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -5295,7 +5311,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Customer ORD-DATA-005</t>
+          <t>Customer ORD-SHIP-EXTRA-005</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -5321,7 +5337,11 @@
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="I101" t="inlineStr"/>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
       <c r="J101" t="inlineStr">
         <is>
           <t>Ravi Kumar</t>
@@ -5807,6 +5827,302 @@
       <c r="J111" t="inlineStr">
         <is>
           <t>Ravi Kumar</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>ORD-INVALID-DISPATCH-NO-ETA</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>2026-10-14 08:00:00</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Customer ORD-NORM-D-001</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>+91 9000000000</t>
+        </is>
+      </c>
+      <c r="E112" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>COD</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>dispatched</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr"/>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>Asha Nair</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>ORD-INVALID-DISPATCH-BAD-ETA</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>2026-10-14 08:00:00</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Customer ORD-NORM-D-001</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>+91 9000000000</t>
+        </is>
+      </c>
+      <c r="E113" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>COD</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>dispatched</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>not-a-date</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>Asha Nair</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>ORD-INVALID-BAD-ORDER-DATE</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>not-a-date</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Customer ORD-NORM-D-001</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>+91 9000000000</t>
+        </is>
+      </c>
+      <c r="E114" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>COD</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>delivered</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>Asha Nair</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>ORD-INVALID-STATUS</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>2026-10-14 08:00:00</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Customer ORD-NORM-D-001</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>+91 9000000000</t>
+        </is>
+      </c>
+      <c r="E115" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>COD</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>in transit</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>Asha Nair</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>ORD-INVALID-PAYMENT</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>2026-10-14 08:00:00</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Customer ORD-NORM-D-001</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>+91 9000000000</t>
+        </is>
+      </c>
+      <c r="E116" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>wallet</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>delivered</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>Asha Nair</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>ORD-INVALID-NEGATIVE-VALUE</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>2026-10-14 08:00:00</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Customer ORD-NORM-D-001</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>+91 9000000000</t>
+        </is>
+      </c>
+      <c r="E117" t="n">
+        <v>-250</v>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>COD</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>delivered</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>Asha Nair</t>
         </is>
       </c>
     </row>

</xml_diff>